<commit_message>
feat: add districtOfBirth dropdown values to dynamic_field seed data
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/dynamic_field.xlsx
+++ b/mosip_master/xlsx/dynamic_field.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="214">
   <si>
     <t>id</t>
   </si>
@@ -200,6 +200,486 @@
   </si>
   <si>
     <t>{"code":"tam","value":"தமிழ்"}</t>
+  </si>
+  <si>
+    <t>10016</t>
+  </si>
+  <si>
+    <t>districtOfBirth</t>
+  </si>
+  <si>
+    <t>District of Birth</t>
+  </si>
+  <si>
+    <t>{"code":"0000","value":"Outside Of Sri Lanka"}</t>
+  </si>
+  <si>
+    <t>10017</t>
+  </si>
+  <si>
+    <t>උපන් දිස්ත්‍රික්කය</t>
+  </si>
+  <si>
+    <t>{"code":"0000","value":"ශ්‍රී ලංකාවෙන් පිට"}</t>
+  </si>
+  <si>
+    <t>10018</t>
+  </si>
+  <si>
+    <t>பிறந்த மாவட்டம்</t>
+  </si>
+  <si>
+    <t>{"code":"0000","value":"இலங்கைக்கு வெளியே"}</t>
+  </si>
+  <si>
+    <t>10019</t>
+  </si>
+  <si>
+    <t>{"code":"0101","value":"Colombo"}</t>
+  </si>
+  <si>
+    <t>10020</t>
+  </si>
+  <si>
+    <t>{"code":"0101","value":"කොළඹ"}</t>
+  </si>
+  <si>
+    <t>10021</t>
+  </si>
+  <si>
+    <t>{"code":"0101","value":"கொழும்பு"}</t>
+  </si>
+  <si>
+    <t>10022</t>
+  </si>
+  <si>
+    <t>{"code":"0102","value":"Gampaha"}</t>
+  </si>
+  <si>
+    <t>10023</t>
+  </si>
+  <si>
+    <t>{"code":"0102","value":"ගම්පහ"}</t>
+  </si>
+  <si>
+    <t>10024</t>
+  </si>
+  <si>
+    <t>{"code":"0102","value":"கம்பஹா"}</t>
+  </si>
+  <si>
+    <t>10025</t>
+  </si>
+  <si>
+    <t>{"code":"0103","value":"Kaluthara"}</t>
+  </si>
+  <si>
+    <t>10026</t>
+  </si>
+  <si>
+    <t>{"code":"0103","value":"කළුතර"}</t>
+  </si>
+  <si>
+    <t>10027</t>
+  </si>
+  <si>
+    <t>{"code":"0103","value":"களுத்துறை"}</t>
+  </si>
+  <si>
+    <t>10028</t>
+  </si>
+  <si>
+    <t>{"code":"0201","value":"Kandy"}</t>
+  </si>
+  <si>
+    <t>10029</t>
+  </si>
+  <si>
+    <t>{"code":"0201","value":"මහනුවර"}</t>
+  </si>
+  <si>
+    <t>10030</t>
+  </si>
+  <si>
+    <t>{"code":"0201","value":"கண்டி"}</t>
+  </si>
+  <si>
+    <t>10031</t>
+  </si>
+  <si>
+    <t>{"code":"0202","value":"Matale"}</t>
+  </si>
+  <si>
+    <t>10032</t>
+  </si>
+  <si>
+    <t>{"code":"0202","value":"මාතලේ"}</t>
+  </si>
+  <si>
+    <t>10033</t>
+  </si>
+  <si>
+    <t>{"code":"0202","value":"மாத்தளை"}</t>
+  </si>
+  <si>
+    <t>10034</t>
+  </si>
+  <si>
+    <t>{"code":"0203","value":"Nuwara Eliya"}</t>
+  </si>
+  <si>
+    <t>10035</t>
+  </si>
+  <si>
+    <t>{"code":"0203","value":"නුවරඑළිය"}</t>
+  </si>
+  <si>
+    <t>10036</t>
+  </si>
+  <si>
+    <t>{"code":"0203","value":"நுவரெலியா"}</t>
+  </si>
+  <si>
+    <t>10037</t>
+  </si>
+  <si>
+    <t>{"code":"0301","value":"Galle"}</t>
+  </si>
+  <si>
+    <t>10038</t>
+  </si>
+  <si>
+    <t>{"code":"0301","value":"ගාල්ල"}</t>
+  </si>
+  <si>
+    <t>10039</t>
+  </si>
+  <si>
+    <t>{"code":"0301","value":"காலி"}</t>
+  </si>
+  <si>
+    <t>10040</t>
+  </si>
+  <si>
+    <t>{"code":"0302","value":"Matara"}</t>
+  </si>
+  <si>
+    <t>10041</t>
+  </si>
+  <si>
+    <t>{"code":"0302","value":"මාතර"}</t>
+  </si>
+  <si>
+    <t>10042</t>
+  </si>
+  <si>
+    <t>{"code":"0302","value":"மாத்தறை"}</t>
+  </si>
+  <si>
+    <t>10043</t>
+  </si>
+  <si>
+    <t>{"code":"0303","value":"Hambantota"}</t>
+  </si>
+  <si>
+    <t>10044</t>
+  </si>
+  <si>
+    <t>{"code":"0303","value":"හම්බන්තොට"}</t>
+  </si>
+  <si>
+    <t>10045</t>
+  </si>
+  <si>
+    <t>{"code":"0303","value":"அம்பாந்தோட்டை"}</t>
+  </si>
+  <si>
+    <t>10046</t>
+  </si>
+  <si>
+    <t>{"code":"0401","value":"Jaffna"}</t>
+  </si>
+  <si>
+    <t>10047</t>
+  </si>
+  <si>
+    <t>{"code":"0401","value":"යාපනය"}</t>
+  </si>
+  <si>
+    <t>10048</t>
+  </si>
+  <si>
+    <t>{"code":"0401","value":"யாழ்ப்பாணம்"}</t>
+  </si>
+  <si>
+    <t>10049</t>
+  </si>
+  <si>
+    <t>{"code":"0402","value":"Mannar"}</t>
+  </si>
+  <si>
+    <t>10050</t>
+  </si>
+  <si>
+    <t>{"code":"0402","value":"මන්නාරම"}</t>
+  </si>
+  <si>
+    <t>10051</t>
+  </si>
+  <si>
+    <t>{"code":"0402","value":"மன்னார்"}</t>
+  </si>
+  <si>
+    <t>10052</t>
+  </si>
+  <si>
+    <t>{"code":"0403","value":"Vavuniya"}</t>
+  </si>
+  <si>
+    <t>10053</t>
+  </si>
+  <si>
+    <t>{"code":"0403","value":"වවුනියාව"}</t>
+  </si>
+  <si>
+    <t>10054</t>
+  </si>
+  <si>
+    <t>{"code":"0403","value":"வவுனியா"}</t>
+  </si>
+  <si>
+    <t>10055</t>
+  </si>
+  <si>
+    <t>{"code":"0404","value":"Mullativu"}</t>
+  </si>
+  <si>
+    <t>10056</t>
+  </si>
+  <si>
+    <t>{"code":"0404","value":"මුලතිව්"}</t>
+  </si>
+  <si>
+    <t>10057</t>
+  </si>
+  <si>
+    <t>{"code":"0404","value":"முல்லைத்தீவு"}</t>
+  </si>
+  <si>
+    <t>10058</t>
+  </si>
+  <si>
+    <t>{"code":"0405","value":"Killinochchi"}</t>
+  </si>
+  <si>
+    <t>10059</t>
+  </si>
+  <si>
+    <t>{"code":"0405","value":"කිලිනොච්චි"}</t>
+  </si>
+  <si>
+    <t>10060</t>
+  </si>
+  <si>
+    <t>{"code":"0405","value":"கிளிநொச்சி"}</t>
+  </si>
+  <si>
+    <t>10061</t>
+  </si>
+  <si>
+    <t>{"code":"0501","value":"Batticaloa"}</t>
+  </si>
+  <si>
+    <t>10062</t>
+  </si>
+  <si>
+    <t>{"code":"0501","value":"මඩකලපුව"}</t>
+  </si>
+  <si>
+    <t>10063</t>
+  </si>
+  <si>
+    <t>{"code":"0501","value":"மட்டக்களப்பு"}</t>
+  </si>
+  <si>
+    <t>10064</t>
+  </si>
+  <si>
+    <t>{"code":"0502","value":"Ampara"}</t>
+  </si>
+  <si>
+    <t>10065</t>
+  </si>
+  <si>
+    <t>{"code":"0502","value":"අම්පාර"}</t>
+  </si>
+  <si>
+    <t>10066</t>
+  </si>
+  <si>
+    <t>{"code":"0502","value":"அம்பாறை"}</t>
+  </si>
+  <si>
+    <t>10067</t>
+  </si>
+  <si>
+    <t>{"code":"0503","value":"Trincomalee"}</t>
+  </si>
+  <si>
+    <t>10068</t>
+  </si>
+  <si>
+    <t>{"code":"0503","value":"ත්‍රිකුණාමලය"}</t>
+  </si>
+  <si>
+    <t>10069</t>
+  </si>
+  <si>
+    <t>{"code":"0503","value":"திருகோணமலை"}</t>
+  </si>
+  <si>
+    <t>10070</t>
+  </si>
+  <si>
+    <t>{"code":"0601","value":"Kurunegala"}</t>
+  </si>
+  <si>
+    <t>10071</t>
+  </si>
+  <si>
+    <t>{"code":"0601","value":"කුරුණෑගල"}</t>
+  </si>
+  <si>
+    <t>10072</t>
+  </si>
+  <si>
+    <t>{"code":"0601","value":"குருநாகல்"}</t>
+  </si>
+  <si>
+    <t>10073</t>
+  </si>
+  <si>
+    <t>{"code":"0602","value":"Puttalam"}</t>
+  </si>
+  <si>
+    <t>10074</t>
+  </si>
+  <si>
+    <t>{"code":"0602","value":"පුත්තලම"}</t>
+  </si>
+  <si>
+    <t>10075</t>
+  </si>
+  <si>
+    <t>{"code":"0602","value":"புத்தளம்"}</t>
+  </si>
+  <si>
+    <t>10076</t>
+  </si>
+  <si>
+    <t>{"code":"0701","value":"Anuradhapura"}</t>
+  </si>
+  <si>
+    <t>10077</t>
+  </si>
+  <si>
+    <t>{"code":"0701","value":"අනුරාධපුරය"}</t>
+  </si>
+  <si>
+    <t>10078</t>
+  </si>
+  <si>
+    <t>{"code":"0701","value":"அனுராதபுரம்"}</t>
+  </si>
+  <si>
+    <t>10079</t>
+  </si>
+  <si>
+    <t>{"code":"0702","value":"Polonnaruwa"}</t>
+  </si>
+  <si>
+    <t>10080</t>
+  </si>
+  <si>
+    <t>{"code":"0702","value":"පොළොන්නරුව"}</t>
+  </si>
+  <si>
+    <t>10081</t>
+  </si>
+  <si>
+    <t>{"code":"0702","value":"பொலன்னறுவை"}</t>
+  </si>
+  <si>
+    <t>10082</t>
+  </si>
+  <si>
+    <t>{"code":"0801","value":"Badulla"}</t>
+  </si>
+  <si>
+    <t>10083</t>
+  </si>
+  <si>
+    <t>{"code":"0801","value":"බදුල්ල"}</t>
+  </si>
+  <si>
+    <t>10084</t>
+  </si>
+  <si>
+    <t>{"code":"0801","value":"பதுளை"}</t>
+  </si>
+  <si>
+    <t>10085</t>
+  </si>
+  <si>
+    <t>{"code":"0802","value":"Monaragala"}</t>
+  </si>
+  <si>
+    <t>10086</t>
+  </si>
+  <si>
+    <t>{"code":"0802","value":"මොණරාගල"}</t>
+  </si>
+  <si>
+    <t>10087</t>
+  </si>
+  <si>
+    <t>{"code":"0802","value":"மொணராகலை"}</t>
+  </si>
+  <si>
+    <t>10088</t>
+  </si>
+  <si>
+    <t>{"code":"0901","value":"Ratnapura"}</t>
+  </si>
+  <si>
+    <t>10089</t>
+  </si>
+  <si>
+    <t>{"code":"0901","value":"රත්නපුර"}</t>
+  </si>
+  <si>
+    <t>10090</t>
+  </si>
+  <si>
+    <t>{"code":"0901","value":"இரத்தினபுரி"}</t>
+  </si>
+  <si>
+    <t>10091</t>
+  </si>
+  <si>
+    <t>{"code":"0902","value":"Kegalle"}</t>
+  </si>
+  <si>
+    <t>10092</t>
+  </si>
+  <si>
+    <t>{"code":"0902","value":"කෑගල්ල"}</t>
+  </si>
+  <si>
+    <t>10093</t>
+  </si>
+  <si>
+    <t>{"code":"0902","value":"கேகாலை"}</t>
   </si>
 </sst>
 </file>
@@ -562,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="27.7109375" customWidth="1"/>
@@ -1032,6 +1512,2268 @@
         <v>17</v>
       </c>
     </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>63</v>
+      </c>
+      <c r="F19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>65</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" t="s">
+        <v>67</v>
+      </c>
+      <c r="F21" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" t="s">
+        <v>69</v>
+      </c>
+      <c r="F22" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" t="s">
+        <v>16</v>
+      </c>
+      <c r="I22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
+        <v>71</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>73</v>
+      </c>
+      <c r="F24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" t="s">
+        <v>62</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" t="s">
+        <v>56</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
+        <v>77</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>79</v>
+      </c>
+      <c r="F27" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>80</v>
+      </c>
+      <c r="B28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>81</v>
+      </c>
+      <c r="F28" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" t="s">
+        <v>16</v>
+      </c>
+      <c r="I29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>84</v>
+      </c>
+      <c r="B30" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
+        <v>85</v>
+      </c>
+      <c r="F30" t="s">
+        <v>21</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" t="s">
+        <v>62</v>
+      </c>
+      <c r="D31" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" t="s">
+        <v>87</v>
+      </c>
+      <c r="F31" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" t="s">
+        <v>89</v>
+      </c>
+      <c r="F32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" t="s">
+        <v>16</v>
+      </c>
+      <c r="I32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>90</v>
+      </c>
+      <c r="B33" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>91</v>
+      </c>
+      <c r="F33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" t="s">
+        <v>62</v>
+      </c>
+      <c r="D34" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" t="s">
+        <v>93</v>
+      </c>
+      <c r="F34" t="s">
+        <v>25</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>94</v>
+      </c>
+      <c r="B35" t="s">
+        <v>55</v>
+      </c>
+      <c r="C35" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>95</v>
+      </c>
+      <c r="F35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" t="s">
+        <v>16</v>
+      </c>
+      <c r="I35" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>96</v>
+      </c>
+      <c r="B36" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" t="s">
+        <v>59</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
+        <v>97</v>
+      </c>
+      <c r="F36" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" t="s">
+        <v>16</v>
+      </c>
+      <c r="I36" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" t="s">
+        <v>62</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" t="s">
+        <v>25</v>
+      </c>
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" t="s">
+        <v>16</v>
+      </c>
+      <c r="I37" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>100</v>
+      </c>
+      <c r="B38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" t="s">
+        <v>101</v>
+      </c>
+      <c r="F38" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I38" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>102</v>
+      </c>
+      <c r="B39" t="s">
+        <v>55</v>
+      </c>
+      <c r="C39" t="s">
+        <v>59</v>
+      </c>
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" t="s">
+        <v>103</v>
+      </c>
+      <c r="F39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" t="s">
+        <v>16</v>
+      </c>
+      <c r="I39" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>104</v>
+      </c>
+      <c r="B40" t="s">
+        <v>55</v>
+      </c>
+      <c r="C40" t="s">
+        <v>62</v>
+      </c>
+      <c r="D40" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" t="s">
+        <v>105</v>
+      </c>
+      <c r="F40" t="s">
+        <v>25</v>
+      </c>
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" t="s">
+        <v>16</v>
+      </c>
+      <c r="I40" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>106</v>
+      </c>
+      <c r="B41" t="s">
+        <v>55</v>
+      </c>
+      <c r="C41" t="s">
+        <v>56</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" t="s">
+        <v>107</v>
+      </c>
+      <c r="F41" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" t="s">
+        <v>16</v>
+      </c>
+      <c r="I41" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>108</v>
+      </c>
+      <c r="B42" t="s">
+        <v>55</v>
+      </c>
+      <c r="C42" t="s">
+        <v>59</v>
+      </c>
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" t="s">
+        <v>109</v>
+      </c>
+      <c r="F42" t="s">
+        <v>21</v>
+      </c>
+      <c r="G42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" t="s">
+        <v>16</v>
+      </c>
+      <c r="I42" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>110</v>
+      </c>
+      <c r="B43" t="s">
+        <v>55</v>
+      </c>
+      <c r="C43" t="s">
+        <v>62</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>111</v>
+      </c>
+      <c r="F43" t="s">
+        <v>25</v>
+      </c>
+      <c r="G43" t="s">
+        <v>15</v>
+      </c>
+      <c r="H43" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>112</v>
+      </c>
+      <c r="B44" t="s">
+        <v>55</v>
+      </c>
+      <c r="C44" t="s">
+        <v>56</v>
+      </c>
+      <c r="D44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E44" t="s">
+        <v>113</v>
+      </c>
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" t="s">
+        <v>15</v>
+      </c>
+      <c r="H44" t="s">
+        <v>16</v>
+      </c>
+      <c r="I44" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>114</v>
+      </c>
+      <c r="B45" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45" t="s">
+        <v>59</v>
+      </c>
+      <c r="D45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45" t="s">
+        <v>115</v>
+      </c>
+      <c r="F45" t="s">
+        <v>21</v>
+      </c>
+      <c r="G45" t="s">
+        <v>15</v>
+      </c>
+      <c r="H45" t="s">
+        <v>16</v>
+      </c>
+      <c r="I45" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>116</v>
+      </c>
+      <c r="B46" t="s">
+        <v>55</v>
+      </c>
+      <c r="C46" t="s">
+        <v>62</v>
+      </c>
+      <c r="D46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E46" t="s">
+        <v>117</v>
+      </c>
+      <c r="F46" t="s">
+        <v>25</v>
+      </c>
+      <c r="G46" t="s">
+        <v>15</v>
+      </c>
+      <c r="H46" t="s">
+        <v>16</v>
+      </c>
+      <c r="I46" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>118</v>
+      </c>
+      <c r="B47" t="s">
+        <v>55</v>
+      </c>
+      <c r="C47" t="s">
+        <v>56</v>
+      </c>
+      <c r="D47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47" t="s">
+        <v>119</v>
+      </c>
+      <c r="F47" t="s">
+        <v>14</v>
+      </c>
+      <c r="G47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" t="s">
+        <v>16</v>
+      </c>
+      <c r="I47" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>120</v>
+      </c>
+      <c r="B48" t="s">
+        <v>55</v>
+      </c>
+      <c r="C48" t="s">
+        <v>59</v>
+      </c>
+      <c r="D48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E48" t="s">
+        <v>121</v>
+      </c>
+      <c r="F48" t="s">
+        <v>21</v>
+      </c>
+      <c r="G48" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" t="s">
+        <v>16</v>
+      </c>
+      <c r="I48" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>122</v>
+      </c>
+      <c r="B49" t="s">
+        <v>55</v>
+      </c>
+      <c r="C49" t="s">
+        <v>62</v>
+      </c>
+      <c r="D49" t="s">
+        <v>12</v>
+      </c>
+      <c r="E49" t="s">
+        <v>123</v>
+      </c>
+      <c r="F49" t="s">
+        <v>25</v>
+      </c>
+      <c r="G49" t="s">
+        <v>15</v>
+      </c>
+      <c r="H49" t="s">
+        <v>16</v>
+      </c>
+      <c r="I49" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>124</v>
+      </c>
+      <c r="B50" t="s">
+        <v>55</v>
+      </c>
+      <c r="C50" t="s">
+        <v>56</v>
+      </c>
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" t="s">
+        <v>125</v>
+      </c>
+      <c r="F50" t="s">
+        <v>14</v>
+      </c>
+      <c r="G50" t="s">
+        <v>15</v>
+      </c>
+      <c r="H50" t="s">
+        <v>16</v>
+      </c>
+      <c r="I50" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>126</v>
+      </c>
+      <c r="B51" t="s">
+        <v>55</v>
+      </c>
+      <c r="C51" t="s">
+        <v>59</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>127</v>
+      </c>
+      <c r="F51" t="s">
+        <v>21</v>
+      </c>
+      <c r="G51" t="s">
+        <v>15</v>
+      </c>
+      <c r="H51" t="s">
+        <v>16</v>
+      </c>
+      <c r="I51" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>128</v>
+      </c>
+      <c r="B52" t="s">
+        <v>55</v>
+      </c>
+      <c r="C52" t="s">
+        <v>62</v>
+      </c>
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" t="s">
+        <v>129</v>
+      </c>
+      <c r="F52" t="s">
+        <v>25</v>
+      </c>
+      <c r="G52" t="s">
+        <v>15</v>
+      </c>
+      <c r="H52" t="s">
+        <v>16</v>
+      </c>
+      <c r="I52" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>130</v>
+      </c>
+      <c r="B53" t="s">
+        <v>55</v>
+      </c>
+      <c r="C53" t="s">
+        <v>56</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>131</v>
+      </c>
+      <c r="F53" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53" t="s">
+        <v>15</v>
+      </c>
+      <c r="H53" t="s">
+        <v>16</v>
+      </c>
+      <c r="I53" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>132</v>
+      </c>
+      <c r="B54" t="s">
+        <v>55</v>
+      </c>
+      <c r="C54" t="s">
+        <v>59</v>
+      </c>
+      <c r="D54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>133</v>
+      </c>
+      <c r="F54" t="s">
+        <v>21</v>
+      </c>
+      <c r="G54" t="s">
+        <v>15</v>
+      </c>
+      <c r="H54" t="s">
+        <v>16</v>
+      </c>
+      <c r="I54" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>134</v>
+      </c>
+      <c r="B55" t="s">
+        <v>55</v>
+      </c>
+      <c r="C55" t="s">
+        <v>62</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>135</v>
+      </c>
+      <c r="F55" t="s">
+        <v>25</v>
+      </c>
+      <c r="G55" t="s">
+        <v>15</v>
+      </c>
+      <c r="H55" t="s">
+        <v>16</v>
+      </c>
+      <c r="I55" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>136</v>
+      </c>
+      <c r="B56" t="s">
+        <v>55</v>
+      </c>
+      <c r="C56" t="s">
+        <v>56</v>
+      </c>
+      <c r="D56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" t="s">
+        <v>137</v>
+      </c>
+      <c r="F56" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" t="s">
+        <v>16</v>
+      </c>
+      <c r="I56" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>138</v>
+      </c>
+      <c r="B57" t="s">
+        <v>55</v>
+      </c>
+      <c r="C57" t="s">
+        <v>59</v>
+      </c>
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" t="s">
+        <v>139</v>
+      </c>
+      <c r="F57" t="s">
+        <v>21</v>
+      </c>
+      <c r="G57" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" t="s">
+        <v>16</v>
+      </c>
+      <c r="I57" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>140</v>
+      </c>
+      <c r="B58" t="s">
+        <v>55</v>
+      </c>
+      <c r="C58" t="s">
+        <v>62</v>
+      </c>
+      <c r="D58" t="s">
+        <v>12</v>
+      </c>
+      <c r="E58" t="s">
+        <v>141</v>
+      </c>
+      <c r="F58" t="s">
+        <v>25</v>
+      </c>
+      <c r="G58" t="s">
+        <v>15</v>
+      </c>
+      <c r="H58" t="s">
+        <v>16</v>
+      </c>
+      <c r="I58" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>142</v>
+      </c>
+      <c r="B59" t="s">
+        <v>55</v>
+      </c>
+      <c r="C59" t="s">
+        <v>56</v>
+      </c>
+      <c r="D59" t="s">
+        <v>12</v>
+      </c>
+      <c r="E59" t="s">
+        <v>143</v>
+      </c>
+      <c r="F59" t="s">
+        <v>14</v>
+      </c>
+      <c r="G59" t="s">
+        <v>15</v>
+      </c>
+      <c r="H59" t="s">
+        <v>16</v>
+      </c>
+      <c r="I59" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>144</v>
+      </c>
+      <c r="B60" t="s">
+        <v>55</v>
+      </c>
+      <c r="C60" t="s">
+        <v>59</v>
+      </c>
+      <c r="D60" t="s">
+        <v>12</v>
+      </c>
+      <c r="E60" t="s">
+        <v>145</v>
+      </c>
+      <c r="F60" t="s">
+        <v>21</v>
+      </c>
+      <c r="G60" t="s">
+        <v>15</v>
+      </c>
+      <c r="H60" t="s">
+        <v>16</v>
+      </c>
+      <c r="I60" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>146</v>
+      </c>
+      <c r="B61" t="s">
+        <v>55</v>
+      </c>
+      <c r="C61" t="s">
+        <v>62</v>
+      </c>
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" t="s">
+        <v>147</v>
+      </c>
+      <c r="F61" t="s">
+        <v>25</v>
+      </c>
+      <c r="G61" t="s">
+        <v>15</v>
+      </c>
+      <c r="H61" t="s">
+        <v>16</v>
+      </c>
+      <c r="I61" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>148</v>
+      </c>
+      <c r="B62" t="s">
+        <v>55</v>
+      </c>
+      <c r="C62" t="s">
+        <v>56</v>
+      </c>
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>149</v>
+      </c>
+      <c r="F62" t="s">
+        <v>14</v>
+      </c>
+      <c r="G62" t="s">
+        <v>15</v>
+      </c>
+      <c r="H62" t="s">
+        <v>16</v>
+      </c>
+      <c r="I62" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>150</v>
+      </c>
+      <c r="B63" t="s">
+        <v>55</v>
+      </c>
+      <c r="C63" t="s">
+        <v>59</v>
+      </c>
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" t="s">
+        <v>151</v>
+      </c>
+      <c r="F63" t="s">
+        <v>21</v>
+      </c>
+      <c r="G63" t="s">
+        <v>15</v>
+      </c>
+      <c r="H63" t="s">
+        <v>16</v>
+      </c>
+      <c r="I63" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>152</v>
+      </c>
+      <c r="B64" t="s">
+        <v>55</v>
+      </c>
+      <c r="C64" t="s">
+        <v>62</v>
+      </c>
+      <c r="D64" t="s">
+        <v>12</v>
+      </c>
+      <c r="E64" t="s">
+        <v>153</v>
+      </c>
+      <c r="F64" t="s">
+        <v>25</v>
+      </c>
+      <c r="G64" t="s">
+        <v>15</v>
+      </c>
+      <c r="H64" t="s">
+        <v>16</v>
+      </c>
+      <c r="I64" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>154</v>
+      </c>
+      <c r="B65" t="s">
+        <v>55</v>
+      </c>
+      <c r="C65" t="s">
+        <v>56</v>
+      </c>
+      <c r="D65" t="s">
+        <v>12</v>
+      </c>
+      <c r="E65" t="s">
+        <v>155</v>
+      </c>
+      <c r="F65" t="s">
+        <v>14</v>
+      </c>
+      <c r="G65" t="s">
+        <v>15</v>
+      </c>
+      <c r="H65" t="s">
+        <v>16</v>
+      </c>
+      <c r="I65" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>156</v>
+      </c>
+      <c r="B66" t="s">
+        <v>55</v>
+      </c>
+      <c r="C66" t="s">
+        <v>59</v>
+      </c>
+      <c r="D66" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" t="s">
+        <v>157</v>
+      </c>
+      <c r="F66" t="s">
+        <v>21</v>
+      </c>
+      <c r="G66" t="s">
+        <v>15</v>
+      </c>
+      <c r="H66" t="s">
+        <v>16</v>
+      </c>
+      <c r="I66" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>158</v>
+      </c>
+      <c r="B67" t="s">
+        <v>55</v>
+      </c>
+      <c r="C67" t="s">
+        <v>62</v>
+      </c>
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67" t="s">
+        <v>159</v>
+      </c>
+      <c r="F67" t="s">
+        <v>25</v>
+      </c>
+      <c r="G67" t="s">
+        <v>15</v>
+      </c>
+      <c r="H67" t="s">
+        <v>16</v>
+      </c>
+      <c r="I67" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>160</v>
+      </c>
+      <c r="B68" t="s">
+        <v>55</v>
+      </c>
+      <c r="C68" t="s">
+        <v>56</v>
+      </c>
+      <c r="D68" t="s">
+        <v>12</v>
+      </c>
+      <c r="E68" t="s">
+        <v>161</v>
+      </c>
+      <c r="F68" t="s">
+        <v>14</v>
+      </c>
+      <c r="G68" t="s">
+        <v>15</v>
+      </c>
+      <c r="H68" t="s">
+        <v>16</v>
+      </c>
+      <c r="I68" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>162</v>
+      </c>
+      <c r="B69" t="s">
+        <v>55</v>
+      </c>
+      <c r="C69" t="s">
+        <v>59</v>
+      </c>
+      <c r="D69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" t="s">
+        <v>163</v>
+      </c>
+      <c r="F69" t="s">
+        <v>21</v>
+      </c>
+      <c r="G69" t="s">
+        <v>15</v>
+      </c>
+      <c r="H69" t="s">
+        <v>16</v>
+      </c>
+      <c r="I69" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>164</v>
+      </c>
+      <c r="B70" t="s">
+        <v>55</v>
+      </c>
+      <c r="C70" t="s">
+        <v>62</v>
+      </c>
+      <c r="D70" t="s">
+        <v>12</v>
+      </c>
+      <c r="E70" t="s">
+        <v>165</v>
+      </c>
+      <c r="F70" t="s">
+        <v>25</v>
+      </c>
+      <c r="G70" t="s">
+        <v>15</v>
+      </c>
+      <c r="H70" t="s">
+        <v>16</v>
+      </c>
+      <c r="I70" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>166</v>
+      </c>
+      <c r="B71" t="s">
+        <v>55</v>
+      </c>
+      <c r="C71" t="s">
+        <v>56</v>
+      </c>
+      <c r="D71" t="s">
+        <v>12</v>
+      </c>
+      <c r="E71" t="s">
+        <v>167</v>
+      </c>
+      <c r="F71" t="s">
+        <v>14</v>
+      </c>
+      <c r="G71" t="s">
+        <v>15</v>
+      </c>
+      <c r="H71" t="s">
+        <v>16</v>
+      </c>
+      <c r="I71" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>168</v>
+      </c>
+      <c r="B72" t="s">
+        <v>55</v>
+      </c>
+      <c r="C72" t="s">
+        <v>59</v>
+      </c>
+      <c r="D72" t="s">
+        <v>12</v>
+      </c>
+      <c r="E72" t="s">
+        <v>169</v>
+      </c>
+      <c r="F72" t="s">
+        <v>21</v>
+      </c>
+      <c r="G72" t="s">
+        <v>15</v>
+      </c>
+      <c r="H72" t="s">
+        <v>16</v>
+      </c>
+      <c r="I72" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>170</v>
+      </c>
+      <c r="B73" t="s">
+        <v>55</v>
+      </c>
+      <c r="C73" t="s">
+        <v>62</v>
+      </c>
+      <c r="D73" t="s">
+        <v>12</v>
+      </c>
+      <c r="E73" t="s">
+        <v>171</v>
+      </c>
+      <c r="F73" t="s">
+        <v>25</v>
+      </c>
+      <c r="G73" t="s">
+        <v>15</v>
+      </c>
+      <c r="H73" t="s">
+        <v>16</v>
+      </c>
+      <c r="I73" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>172</v>
+      </c>
+      <c r="B74" t="s">
+        <v>55</v>
+      </c>
+      <c r="C74" t="s">
+        <v>56</v>
+      </c>
+      <c r="D74" t="s">
+        <v>12</v>
+      </c>
+      <c r="E74" t="s">
+        <v>173</v>
+      </c>
+      <c r="F74" t="s">
+        <v>14</v>
+      </c>
+      <c r="G74" t="s">
+        <v>15</v>
+      </c>
+      <c r="H74" t="s">
+        <v>16</v>
+      </c>
+      <c r="I74" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>174</v>
+      </c>
+      <c r="B75" t="s">
+        <v>55</v>
+      </c>
+      <c r="C75" t="s">
+        <v>59</v>
+      </c>
+      <c r="D75" t="s">
+        <v>12</v>
+      </c>
+      <c r="E75" t="s">
+        <v>175</v>
+      </c>
+      <c r="F75" t="s">
+        <v>21</v>
+      </c>
+      <c r="G75" t="s">
+        <v>15</v>
+      </c>
+      <c r="H75" t="s">
+        <v>16</v>
+      </c>
+      <c r="I75" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>176</v>
+      </c>
+      <c r="B76" t="s">
+        <v>55</v>
+      </c>
+      <c r="C76" t="s">
+        <v>62</v>
+      </c>
+      <c r="D76" t="s">
+        <v>12</v>
+      </c>
+      <c r="E76" t="s">
+        <v>177</v>
+      </c>
+      <c r="F76" t="s">
+        <v>25</v>
+      </c>
+      <c r="G76" t="s">
+        <v>15</v>
+      </c>
+      <c r="H76" t="s">
+        <v>16</v>
+      </c>
+      <c r="I76" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>178</v>
+      </c>
+      <c r="B77" t="s">
+        <v>55</v>
+      </c>
+      <c r="C77" t="s">
+        <v>56</v>
+      </c>
+      <c r="D77" t="s">
+        <v>12</v>
+      </c>
+      <c r="E77" t="s">
+        <v>179</v>
+      </c>
+      <c r="F77" t="s">
+        <v>14</v>
+      </c>
+      <c r="G77" t="s">
+        <v>15</v>
+      </c>
+      <c r="H77" t="s">
+        <v>16</v>
+      </c>
+      <c r="I77" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>180</v>
+      </c>
+      <c r="B78" t="s">
+        <v>55</v>
+      </c>
+      <c r="C78" t="s">
+        <v>59</v>
+      </c>
+      <c r="D78" t="s">
+        <v>12</v>
+      </c>
+      <c r="E78" t="s">
+        <v>181</v>
+      </c>
+      <c r="F78" t="s">
+        <v>21</v>
+      </c>
+      <c r="G78" t="s">
+        <v>15</v>
+      </c>
+      <c r="H78" t="s">
+        <v>16</v>
+      </c>
+      <c r="I78" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>182</v>
+      </c>
+      <c r="B79" t="s">
+        <v>55</v>
+      </c>
+      <c r="C79" t="s">
+        <v>62</v>
+      </c>
+      <c r="D79" t="s">
+        <v>12</v>
+      </c>
+      <c r="E79" t="s">
+        <v>183</v>
+      </c>
+      <c r="F79" t="s">
+        <v>25</v>
+      </c>
+      <c r="G79" t="s">
+        <v>15</v>
+      </c>
+      <c r="H79" t="s">
+        <v>16</v>
+      </c>
+      <c r="I79" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>184</v>
+      </c>
+      <c r="B80" t="s">
+        <v>55</v>
+      </c>
+      <c r="C80" t="s">
+        <v>56</v>
+      </c>
+      <c r="D80" t="s">
+        <v>12</v>
+      </c>
+      <c r="E80" t="s">
+        <v>185</v>
+      </c>
+      <c r="F80" t="s">
+        <v>14</v>
+      </c>
+      <c r="G80" t="s">
+        <v>15</v>
+      </c>
+      <c r="H80" t="s">
+        <v>16</v>
+      </c>
+      <c r="I80" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>186</v>
+      </c>
+      <c r="B81" t="s">
+        <v>55</v>
+      </c>
+      <c r="C81" t="s">
+        <v>59</v>
+      </c>
+      <c r="D81" t="s">
+        <v>12</v>
+      </c>
+      <c r="E81" t="s">
+        <v>187</v>
+      </c>
+      <c r="F81" t="s">
+        <v>21</v>
+      </c>
+      <c r="G81" t="s">
+        <v>15</v>
+      </c>
+      <c r="H81" t="s">
+        <v>16</v>
+      </c>
+      <c r="I81" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>188</v>
+      </c>
+      <c r="B82" t="s">
+        <v>55</v>
+      </c>
+      <c r="C82" t="s">
+        <v>62</v>
+      </c>
+      <c r="D82" t="s">
+        <v>12</v>
+      </c>
+      <c r="E82" t="s">
+        <v>189</v>
+      </c>
+      <c r="F82" t="s">
+        <v>25</v>
+      </c>
+      <c r="G82" t="s">
+        <v>15</v>
+      </c>
+      <c r="H82" t="s">
+        <v>16</v>
+      </c>
+      <c r="I82" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>190</v>
+      </c>
+      <c r="B83" t="s">
+        <v>55</v>
+      </c>
+      <c r="C83" t="s">
+        <v>56</v>
+      </c>
+      <c r="D83" t="s">
+        <v>12</v>
+      </c>
+      <c r="E83" t="s">
+        <v>191</v>
+      </c>
+      <c r="F83" t="s">
+        <v>14</v>
+      </c>
+      <c r="G83" t="s">
+        <v>15</v>
+      </c>
+      <c r="H83" t="s">
+        <v>16</v>
+      </c>
+      <c r="I83" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>192</v>
+      </c>
+      <c r="B84" t="s">
+        <v>55</v>
+      </c>
+      <c r="C84" t="s">
+        <v>59</v>
+      </c>
+      <c r="D84" t="s">
+        <v>12</v>
+      </c>
+      <c r="E84" t="s">
+        <v>193</v>
+      </c>
+      <c r="F84" t="s">
+        <v>21</v>
+      </c>
+      <c r="G84" t="s">
+        <v>15</v>
+      </c>
+      <c r="H84" t="s">
+        <v>16</v>
+      </c>
+      <c r="I84" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>194</v>
+      </c>
+      <c r="B85" t="s">
+        <v>55</v>
+      </c>
+      <c r="C85" t="s">
+        <v>62</v>
+      </c>
+      <c r="D85" t="s">
+        <v>12</v>
+      </c>
+      <c r="E85" t="s">
+        <v>195</v>
+      </c>
+      <c r="F85" t="s">
+        <v>25</v>
+      </c>
+      <c r="G85" t="s">
+        <v>15</v>
+      </c>
+      <c r="H85" t="s">
+        <v>16</v>
+      </c>
+      <c r="I85" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>196</v>
+      </c>
+      <c r="B86" t="s">
+        <v>55</v>
+      </c>
+      <c r="C86" t="s">
+        <v>56</v>
+      </c>
+      <c r="D86" t="s">
+        <v>12</v>
+      </c>
+      <c r="E86" t="s">
+        <v>197</v>
+      </c>
+      <c r="F86" t="s">
+        <v>14</v>
+      </c>
+      <c r="G86" t="s">
+        <v>15</v>
+      </c>
+      <c r="H86" t="s">
+        <v>16</v>
+      </c>
+      <c r="I86" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>198</v>
+      </c>
+      <c r="B87" t="s">
+        <v>55</v>
+      </c>
+      <c r="C87" t="s">
+        <v>59</v>
+      </c>
+      <c r="D87" t="s">
+        <v>12</v>
+      </c>
+      <c r="E87" t="s">
+        <v>199</v>
+      </c>
+      <c r="F87" t="s">
+        <v>21</v>
+      </c>
+      <c r="G87" t="s">
+        <v>15</v>
+      </c>
+      <c r="H87" t="s">
+        <v>16</v>
+      </c>
+      <c r="I87" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>200</v>
+      </c>
+      <c r="B88" t="s">
+        <v>55</v>
+      </c>
+      <c r="C88" t="s">
+        <v>62</v>
+      </c>
+      <c r="D88" t="s">
+        <v>12</v>
+      </c>
+      <c r="E88" t="s">
+        <v>201</v>
+      </c>
+      <c r="F88" t="s">
+        <v>25</v>
+      </c>
+      <c r="G88" t="s">
+        <v>15</v>
+      </c>
+      <c r="H88" t="s">
+        <v>16</v>
+      </c>
+      <c r="I88" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>202</v>
+      </c>
+      <c r="B89" t="s">
+        <v>55</v>
+      </c>
+      <c r="C89" t="s">
+        <v>56</v>
+      </c>
+      <c r="D89" t="s">
+        <v>12</v>
+      </c>
+      <c r="E89" t="s">
+        <v>203</v>
+      </c>
+      <c r="F89" t="s">
+        <v>14</v>
+      </c>
+      <c r="G89" t="s">
+        <v>15</v>
+      </c>
+      <c r="H89" t="s">
+        <v>16</v>
+      </c>
+      <c r="I89" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>204</v>
+      </c>
+      <c r="B90" t="s">
+        <v>55</v>
+      </c>
+      <c r="C90" t="s">
+        <v>59</v>
+      </c>
+      <c r="D90" t="s">
+        <v>12</v>
+      </c>
+      <c r="E90" t="s">
+        <v>205</v>
+      </c>
+      <c r="F90" t="s">
+        <v>21</v>
+      </c>
+      <c r="G90" t="s">
+        <v>15</v>
+      </c>
+      <c r="H90" t="s">
+        <v>16</v>
+      </c>
+      <c r="I90" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>206</v>
+      </c>
+      <c r="B91" t="s">
+        <v>55</v>
+      </c>
+      <c r="C91" t="s">
+        <v>62</v>
+      </c>
+      <c r="D91" t="s">
+        <v>12</v>
+      </c>
+      <c r="E91" t="s">
+        <v>207</v>
+      </c>
+      <c r="F91" t="s">
+        <v>25</v>
+      </c>
+      <c r="G91" t="s">
+        <v>15</v>
+      </c>
+      <c r="H91" t="s">
+        <v>16</v>
+      </c>
+      <c r="I91" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>208</v>
+      </c>
+      <c r="B92" t="s">
+        <v>55</v>
+      </c>
+      <c r="C92" t="s">
+        <v>56</v>
+      </c>
+      <c r="D92" t="s">
+        <v>12</v>
+      </c>
+      <c r="E92" t="s">
+        <v>209</v>
+      </c>
+      <c r="F92" t="s">
+        <v>14</v>
+      </c>
+      <c r="G92" t="s">
+        <v>15</v>
+      </c>
+      <c r="H92" t="s">
+        <v>16</v>
+      </c>
+      <c r="I92" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>210</v>
+      </c>
+      <c r="B93" t="s">
+        <v>55</v>
+      </c>
+      <c r="C93" t="s">
+        <v>59</v>
+      </c>
+      <c r="D93" t="s">
+        <v>12</v>
+      </c>
+      <c r="E93" t="s">
+        <v>211</v>
+      </c>
+      <c r="F93" t="s">
+        <v>21</v>
+      </c>
+      <c r="G93" t="s">
+        <v>15</v>
+      </c>
+      <c r="H93" t="s">
+        <v>16</v>
+      </c>
+      <c r="I93" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>212</v>
+      </c>
+      <c r="B94" t="s">
+        <v>55</v>
+      </c>
+      <c r="C94" t="s">
+        <v>62</v>
+      </c>
+      <c r="D94" t="s">
+        <v>12</v>
+      </c>
+      <c r="E94" t="s">
+        <v>213</v>
+      </c>
+      <c r="F94" t="s">
+        <v>25</v>
+      </c>
+      <c r="G94" t="s">
+        <v>15</v>
+      </c>
+      <c r="H94" t="s">
+        <v>16</v>
+      </c>
+      <c r="I94" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: deactivate Outside Of Sri Lanka in the location and District of Birth seed data
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/dynamic_field.xlsx
+++ b/mosip_master/xlsx/dynamic_field.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="215">
   <si>
     <t>id</t>
   </si>
@@ -680,6 +680,9 @@
   </si>
   <si>
     <t>{"code":"0902","value":"கேகாலை"}</t>
+  </si>
+  <si>
+    <t>FALSE</t>
   </si>
 </sst>
 </file>
@@ -1532,7 +1535,7 @@
         <v>14</v>
       </c>
       <c r="G17" t="s">
-        <v>15</v>
+        <v>214</v>
       </c>
       <c r="H17" t="s">
         <v>16</v>
@@ -1561,7 +1564,7 @@
         <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>15</v>
+        <v>214</v>
       </c>
       <c r="H18" t="s">
         <v>16</v>
@@ -1590,7 +1593,7 @@
         <v>25</v>
       </c>
       <c r="G19" t="s">
-        <v>15</v>
+        <v>214</v>
       </c>
       <c r="H19" t="s">
         <v>16</v>

</xml_diff>